<commit_message>
added 3 project ideas
</commit_message>
<xml_diff>
--- a/Submissions/Group Formation/STA380GroupForm.xlsx
+++ b/Submissions/Group Formation/STA380GroupForm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khoig\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christianjasonsumitro/Documents/UTM/STA380/STA380-Project/Submissions/Group Formation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA343530-63AC-4DF9-A11B-418425144C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1A2C62-97A3-9B4D-9A80-A77054FAC55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -118,34 +118,6 @@
     <t>Exponential Distribution</t>
   </si>
   <si>
-    <r>
-      <t>1. Comparison Graph:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t> Overlay a histogram of the simulated data with the theoretical Probability Density Function (PDF) curve.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2. Statistical Validation:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t> Output a table comparing the simulated sample mean and variance against the theoretical formulas.</t>
-    </r>
-  </si>
-  <si>
     <t>Oluwaseye Edwards</t>
   </si>
   <si>
@@ -168,6 +140,24 @@
   </si>
   <si>
     <t>https://github.com/khoigiaho</t>
+  </si>
+  <si>
+    <t>Convolution</t>
+  </si>
+  <si>
+    <t>the sum of i.i.d. squared Gaussians follow a chi-square distribution</t>
+  </si>
+  <si>
+    <t>1. Comparison Graph: Overlay a histogram of the simulated data with the theoretical Probability Density Function (PDF) curve.</t>
+  </si>
+  <si>
+    <t>2. Statistical Validation: Output a table comparing the simulated sample mean and variance against the theoretical formulas.</t>
+  </si>
+  <si>
+    <t>Acceptance-Rejection Method</t>
+  </si>
+  <si>
+    <t>Beta distribution using uniform distribution for g(x)</t>
   </si>
 </sst>
 </file>
@@ -213,31 +203,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <u/>
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF343A40"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -265,7 +255,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -274,10 +264,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -498,17 +488,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="31.7109375" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -516,12 +506,12 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -529,81 +519,97 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3"/>
-      <c r="B8" s="8"/>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3"/>
-      <c r="B9" s="8"/>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="7"/>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="8"/>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3"/>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="8"/>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3"/>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="8"/>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="8"/>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -621,7 +627,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>13</v>
       </c>
@@ -641,7 +647,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>14</v>
       </c>
@@ -661,67 +667,67 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D23">
         <v>1009840273</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D24">
         <v>1007938396</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F24" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
changed ideas 2 & 3
</commit_message>
<xml_diff>
--- a/Submissions/Group Formation/STA380GroupForm.xlsx
+++ b/Submissions/Group Formation/STA380GroupForm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christianjasonsumitro/Documents/UTM/STA380/STA380-Project/Submissions/Group Formation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1A2C62-97A3-9B4D-9A80-A77054FAC55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B078C0DD-0725-1C4C-BACD-6D48ED0E98FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -142,12 +142,6 @@
     <t>https://github.com/khoigiaho</t>
   </si>
   <si>
-    <t>Convolution</t>
-  </si>
-  <si>
-    <t>the sum of i.i.d. squared Gaussians follow a chi-square distribution</t>
-  </si>
-  <si>
     <t>1. Comparison Graph: Overlay a histogram of the simulated data with the theoretical Probability Density Function (PDF) curve.</t>
   </si>
   <si>
@@ -157,7 +151,19 @@
     <t>Acceptance-Rejection Method</t>
   </si>
   <si>
-    <t>Beta distribution using uniform distribution for g(x)</t>
+    <t>Poisson Binomial Distribution</t>
+  </si>
+  <si>
+    <t>Poisson binomial distribution is the discrete probability distribution of a sum of independent Bernoulli trials that are not necessarily identically distributed</t>
+  </si>
+  <si>
+    <t>Mixture</t>
+  </si>
+  <si>
+    <t>k - point Gaussian Distribution</t>
+  </si>
+  <si>
+    <t>One real life example is adult height across different regions</t>
   </si>
 </sst>
 </file>
@@ -540,13 +546,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3"/>
       <c r="B8" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -558,7 +564,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -566,14 +572,16 @@
         <v>4</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="8"/>
+      <c r="B12" s="8" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3"/>
@@ -588,7 +596,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -596,14 +604,16 @@
         <v>4</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="8"/>
+      <c r="B17" s="8" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3"/>

</xml_diff>